<commit_message>
feat(TASA): rediseña ficha como tasa objetivo de política monetaria.
- Construye policy_decisions a partir del calendario de Banxico + serie diaria SIE.
- Separa tasa vigente, última decisión, último ajuste y próxima decisión.
- Renombra visible: TASA OBJETIVO, nombre oficial y aclaración TIIE.
- Elimina "cambio diario" y máximo/mínimo como KPIs principales.
- Sparkline y gráfica usan régimen de tasa (step chart), no repetición diaria.
- Tabla frontend: histórico de decisiones con enlace a comunicado.
- Excel: hojas Serie diaria y Decisiones.
- Botón BOLETÍN se muestra COMUNICADO y abre el último anuncio.
- Tests específicos para TASA.

Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/downloads/indicadores/EMOE/EMOE_datos.xlsx
+++ b/downloads/indicadores/EMOE/EMOE_datos.xlsx
@@ -504,7 +504,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>URL del boletín / serie: https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf · Fecha de publicación: 3 de agosto de 2026</t>
+          <t>URL del boletín / serie: https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf · Fecha de publicación: 1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -577,12 +577,12 @@
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -613,12 +613,12 @@
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H7" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -649,12 +649,12 @@
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -685,12 +685,12 @@
       </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H9" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -721,12 +721,12 @@
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -757,12 +757,12 @@
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H11" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -793,12 +793,12 @@
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -829,12 +829,12 @@
       </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H13" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -865,12 +865,12 @@
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -901,12 +901,12 @@
       </c>
       <c r="G15" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H15" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -937,12 +937,12 @@
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -973,12 +973,12 @@
       </c>
       <c r="G17" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H17" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -1009,12 +1009,12 @@
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H18" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -1045,12 +1045,12 @@
       </c>
       <c r="G19" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H19" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -1081,12 +1081,12 @@
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -1117,12 +1117,12 @@
       </c>
       <c r="G21" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H21" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -1153,12 +1153,12 @@
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H22" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -1189,12 +1189,12 @@
       </c>
       <c r="G23" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H23" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -1225,12 +1225,12 @@
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H24" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -1261,12 +1261,12 @@
       </c>
       <c r="G25" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H25" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -1297,12 +1297,12 @@
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H26" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -1333,12 +1333,12 @@
       </c>
       <c r="G27" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H27" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -1369,12 +1369,12 @@
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H28" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -1405,12 +1405,12 @@
       </c>
       <c r="G29" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H29" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -1441,12 +1441,12 @@
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H30" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -1477,12 +1477,12 @@
       </c>
       <c r="G31" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H31" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -1513,12 +1513,12 @@
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -1549,12 +1549,12 @@
       </c>
       <c r="G33" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H33" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -1585,12 +1585,12 @@
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H34" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -1621,12 +1621,12 @@
       </c>
       <c r="G35" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H35" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -1657,12 +1657,12 @@
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H36" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -1693,12 +1693,12 @@
       </c>
       <c r="G37" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H37" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -1729,12 +1729,12 @@
       </c>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H38" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -1765,12 +1765,12 @@
       </c>
       <c r="G39" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H39" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -1801,12 +1801,12 @@
       </c>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H40" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -1837,12 +1837,12 @@
       </c>
       <c r="G41" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H41" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -1873,12 +1873,12 @@
       </c>
       <c r="G42" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H42" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -1909,12 +1909,12 @@
       </c>
       <c r="G43" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H43" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -1945,12 +1945,12 @@
       </c>
       <c r="G44" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H44" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -1981,12 +1981,12 @@
       </c>
       <c r="G45" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H45" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -2017,12 +2017,12 @@
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H46" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -2053,12 +2053,12 @@
       </c>
       <c r="G47" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H47" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -2089,12 +2089,12 @@
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H48" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -2125,12 +2125,12 @@
       </c>
       <c r="G49" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H49" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -2161,12 +2161,12 @@
       </c>
       <c r="G50" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H50" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -2197,12 +2197,12 @@
       </c>
       <c r="G51" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H51" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -2233,12 +2233,12 @@
       </c>
       <c r="G52" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H52" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -2269,12 +2269,12 @@
       </c>
       <c r="G53" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H53" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -2305,12 +2305,12 @@
       </c>
       <c r="G54" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H54" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -2341,12 +2341,12 @@
       </c>
       <c r="G55" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H55" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -2377,12 +2377,12 @@
       </c>
       <c r="G56" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H56" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -2413,12 +2413,12 @@
       </c>
       <c r="G57" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H57" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -2449,12 +2449,12 @@
       </c>
       <c r="G58" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H58" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -2485,12 +2485,12 @@
       </c>
       <c r="G59" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H59" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -2521,12 +2521,12 @@
       </c>
       <c r="G60" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H60" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -2557,12 +2557,12 @@
       </c>
       <c r="G61" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H61" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -2593,12 +2593,12 @@
       </c>
       <c r="G62" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H62" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -2629,12 +2629,12 @@
       </c>
       <c r="G63" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H63" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -2665,12 +2665,12 @@
       </c>
       <c r="G64" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H64" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -2701,12 +2701,12 @@
       </c>
       <c r="G65" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H65" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -2737,12 +2737,12 @@
       </c>
       <c r="G66" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H66" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -2773,12 +2773,12 @@
       </c>
       <c r="G67" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H67" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -2809,12 +2809,12 @@
       </c>
       <c r="G68" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H68" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -2845,12 +2845,12 @@
       </c>
       <c r="G69" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H69" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -2881,12 +2881,12 @@
       </c>
       <c r="G70" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H70" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -2917,12 +2917,12 @@
       </c>
       <c r="G71" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H71" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -2953,12 +2953,12 @@
       </c>
       <c r="G72" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H72" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -2989,12 +2989,12 @@
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H73" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -3025,12 +3025,12 @@
       </c>
       <c r="G74" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H74" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -3061,12 +3061,12 @@
       </c>
       <c r="G75" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H75" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -3097,12 +3097,12 @@
       </c>
       <c r="G76" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H76" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -3133,12 +3133,12 @@
       </c>
       <c r="G77" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H77" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -3169,12 +3169,12 @@
       </c>
       <c r="G78" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H78" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -3205,12 +3205,12 @@
       </c>
       <c r="G79" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H79" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -3241,12 +3241,12 @@
       </c>
       <c r="G80" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H80" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -3277,12 +3277,12 @@
       </c>
       <c r="G81" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H81" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -3313,12 +3313,12 @@
       </c>
       <c r="G82" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H82" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -3349,12 +3349,12 @@
       </c>
       <c r="G83" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H83" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -3385,12 +3385,12 @@
       </c>
       <c r="G84" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H84" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -3421,12 +3421,12 @@
       </c>
       <c r="G85" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H85" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -3457,12 +3457,12 @@
       </c>
       <c r="G86" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H86" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -3493,12 +3493,12 @@
       </c>
       <c r="G87" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H87" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -3529,12 +3529,12 @@
       </c>
       <c r="G88" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H88" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -3565,12 +3565,12 @@
       </c>
       <c r="G89" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H89" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -3601,12 +3601,12 @@
       </c>
       <c r="G90" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H90" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -3637,12 +3637,12 @@
       </c>
       <c r="G91" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H91" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -3673,12 +3673,12 @@
       </c>
       <c r="G92" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H92" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -3709,12 +3709,12 @@
       </c>
       <c r="G93" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H93" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -3745,12 +3745,12 @@
       </c>
       <c r="G94" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H94" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -3781,12 +3781,12 @@
       </c>
       <c r="G95" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H95" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -3817,12 +3817,12 @@
       </c>
       <c r="G96" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H96" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -3853,12 +3853,12 @@
       </c>
       <c r="G97" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H97" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -3889,12 +3889,12 @@
       </c>
       <c r="G98" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H98" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -3925,12 +3925,12 @@
       </c>
       <c r="G99" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H99" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -3961,12 +3961,12 @@
       </c>
       <c r="G100" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H100" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -3997,12 +3997,12 @@
       </c>
       <c r="G101" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H101" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -4033,12 +4033,12 @@
       </c>
       <c r="G102" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H102" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -4069,12 +4069,12 @@
       </c>
       <c r="G103" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H103" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -4105,12 +4105,12 @@
       </c>
       <c r="G104" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H104" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -4141,12 +4141,12 @@
       </c>
       <c r="G105" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H105" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -4177,12 +4177,12 @@
       </c>
       <c r="G106" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H106" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -4213,12 +4213,12 @@
       </c>
       <c r="G107" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H107" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -4249,12 +4249,12 @@
       </c>
       <c r="G108" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H108" s="7" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>
@@ -4285,12 +4285,12 @@
       </c>
       <c r="G109" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_08.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/ee/ee2026_09.pdf</t>
         </is>
       </c>
       <c r="H109" s="9" t="inlineStr">
         <is>
-          <t>3 de agosto de 2026</t>
+          <t>1 de septiembre de 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(EMOE): confirma IDs BIE de los sectores del ICE.
Incorpora las series oficiales del BIE para los Indicadores de Confianza
Empresarial (ICE) por sector:

- IGOEC: 701401
- Manufacturas: 701570
- Construcción: 701407
- Comercio: 701826
- Servicios privados no financieros: 701975

Actualiza config/series.json, elimina el duplicado de EMOE en
config/indicadores_meta.json y regenera los artefactos de datos y Excel.

Se validaron con build_data, build_excel, pytest y validate.py.

Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/downloads/indicadores/EMOE/EMOE_datos.xlsx
+++ b/downloads/indicadores/EMOE/EMOE_datos.xlsx
@@ -596,10 +596,18 @@
         <v>-0.848</v>
       </c>
       <c r="E6" s="6" t="n"/>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="6" t="n"/>
-      <c r="H6" s="6" t="n"/>
-      <c r="I6" s="6" t="n"/>
+      <c r="F6" s="6" t="n">
+        <v>50.144</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>44.558</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>53.414</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>46.668</v>
+      </c>
       <c r="J6" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -637,10 +645,18 @@
         <v>0.122</v>
       </c>
       <c r="E7" s="8" t="n"/>
-      <c r="F7" s="8" t="n"/>
-      <c r="G7" s="8" t="n"/>
-      <c r="H7" s="8" t="n"/>
-      <c r="I7" s="8" t="n"/>
+      <c r="F7" s="8" t="n">
+        <v>51.009</v>
+      </c>
+      <c r="G7" s="8" t="n">
+        <v>45.309</v>
+      </c>
+      <c r="H7" s="8" t="n">
+        <v>52.681</v>
+      </c>
+      <c r="I7" s="8" t="n">
+        <v>46.759</v>
+      </c>
       <c r="J7" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -678,10 +694,18 @@
         <v>0.92</v>
       </c>
       <c r="E8" s="6" t="n"/>
-      <c r="F8" s="6" t="n"/>
-      <c r="G8" s="6" t="n"/>
-      <c r="H8" s="6" t="n"/>
-      <c r="I8" s="6" t="n"/>
+      <c r="F8" s="6" t="n">
+        <v>51.97</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>46.026</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>54.572</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>47.205</v>
+      </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -719,10 +743,18 @@
         <v>0.003</v>
       </c>
       <c r="E9" s="8" t="n"/>
-      <c r="F9" s="8" t="n"/>
-      <c r="G9" s="8" t="n"/>
-      <c r="H9" s="8" t="n"/>
-      <c r="I9" s="8" t="n"/>
+      <c r="F9" s="8" t="n">
+        <v>52.008</v>
+      </c>
+      <c r="G9" s="8" t="n">
+        <v>46.648</v>
+      </c>
+      <c r="H9" s="8" t="n">
+        <v>53.229</v>
+      </c>
+      <c r="I9" s="8" t="n">
+        <v>47.753</v>
+      </c>
       <c r="J9" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -760,10 +792,18 @@
         <v>-0.855</v>
       </c>
       <c r="E10" s="6" t="n"/>
-      <c r="F10" s="6" t="n"/>
-      <c r="G10" s="6" t="n"/>
-      <c r="H10" s="6" t="n"/>
-      <c r="I10" s="6" t="n"/>
+      <c r="F10" s="6" t="n">
+        <v>50.967</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>46.858</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>52.22</v>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>46.847</v>
+      </c>
       <c r="J10" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -801,10 +841,18 @@
         <v>-0.778</v>
       </c>
       <c r="E11" s="8" t="n"/>
-      <c r="F11" s="8" t="n"/>
-      <c r="G11" s="8" t="n"/>
-      <c r="H11" s="8" t="n"/>
-      <c r="I11" s="8" t="n"/>
+      <c r="F11" s="8" t="n">
+        <v>49.936</v>
+      </c>
+      <c r="G11" s="8" t="n">
+        <v>45.746</v>
+      </c>
+      <c r="H11" s="8" t="n">
+        <v>52.573</v>
+      </c>
+      <c r="I11" s="8" t="n">
+        <v>45.677</v>
+      </c>
       <c r="J11" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -842,10 +890,18 @@
         <v>4.354</v>
       </c>
       <c r="E12" s="6" t="n"/>
-      <c r="F12" s="6" t="n"/>
-      <c r="G12" s="6" t="n"/>
-      <c r="H12" s="6" t="n"/>
-      <c r="I12" s="6" t="n"/>
+      <c r="F12" s="6" t="n">
+        <v>53.001</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>50.325</v>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>56.46</v>
+      </c>
+      <c r="I12" s="6" t="n">
+        <v>50.816</v>
+      </c>
       <c r="J12" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -883,10 +939,18 @@
         <v>0.654</v>
       </c>
       <c r="E13" s="8" t="n"/>
-      <c r="F13" s="8" t="n"/>
-      <c r="G13" s="8" t="n"/>
-      <c r="H13" s="8" t="n"/>
-      <c r="I13" s="8" t="n"/>
+      <c r="F13" s="8" t="n">
+        <v>53.226</v>
+      </c>
+      <c r="G13" s="8" t="n">
+        <v>51.509</v>
+      </c>
+      <c r="H13" s="8" t="n">
+        <v>56.865</v>
+      </c>
+      <c r="I13" s="8" t="n">
+        <v>51.688</v>
+      </c>
       <c r="J13" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -924,10 +988,18 @@
         <v>-1.141</v>
       </c>
       <c r="E14" s="6" t="n"/>
-      <c r="F14" s="6" t="n"/>
-      <c r="G14" s="6" t="n"/>
-      <c r="H14" s="6" t="n"/>
-      <c r="I14" s="6" t="n"/>
+      <c r="F14" s="6" t="n">
+        <v>52.794</v>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>50.06</v>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>55.91</v>
+      </c>
+      <c r="I14" s="6" t="n">
+        <v>50.189</v>
+      </c>
       <c r="J14" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -965,10 +1037,18 @@
         <v>-0.496</v>
       </c>
       <c r="E15" s="8" t="n"/>
-      <c r="F15" s="8" t="n"/>
-      <c r="G15" s="8" t="n"/>
-      <c r="H15" s="8" t="n"/>
-      <c r="I15" s="8" t="n"/>
+      <c r="F15" s="8" t="n">
+        <v>52.278</v>
+      </c>
+      <c r="G15" s="8" t="n">
+        <v>49.549</v>
+      </c>
+      <c r="H15" s="8" t="n">
+        <v>54.93</v>
+      </c>
+      <c r="I15" s="8" t="n">
+        <v>49.952</v>
+      </c>
       <c r="J15" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1006,10 +1086,18 @@
         <v>-1.464</v>
       </c>
       <c r="E16" s="6" t="n"/>
-      <c r="F16" s="6" t="n"/>
-      <c r="G16" s="6" t="n"/>
-      <c r="H16" s="6" t="n"/>
-      <c r="I16" s="6" t="n"/>
+      <c r="F16" s="6" t="n">
+        <v>50.975</v>
+      </c>
+      <c r="G16" s="6" t="n">
+        <v>47.584</v>
+      </c>
+      <c r="H16" s="6" t="n">
+        <v>53.675</v>
+      </c>
+      <c r="I16" s="6" t="n">
+        <v>48.407</v>
+      </c>
       <c r="J16" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1047,10 +1135,18 @@
         <v>0.555</v>
       </c>
       <c r="E17" s="8" t="n"/>
-      <c r="F17" s="8" t="n"/>
-      <c r="G17" s="8" t="n"/>
-      <c r="H17" s="8" t="n"/>
-      <c r="I17" s="8" t="n"/>
+      <c r="F17" s="8" t="n">
+        <v>51.004</v>
+      </c>
+      <c r="G17" s="8" t="n">
+        <v>48.358</v>
+      </c>
+      <c r="H17" s="8" t="n">
+        <v>54.717</v>
+      </c>
+      <c r="I17" s="8" t="n">
+        <v>48.912</v>
+      </c>
       <c r="J17" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1090,10 +1186,18 @@
       <c r="E18" s="6" t="n">
         <v>3.286</v>
       </c>
-      <c r="F18" s="6" t="n"/>
-      <c r="G18" s="6" t="n"/>
-      <c r="H18" s="6" t="n"/>
-      <c r="I18" s="6" t="n"/>
+      <c r="F18" s="6" t="n">
+        <v>52.962</v>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>47.435</v>
+      </c>
+      <c r="H18" s="6" t="n">
+        <v>54.194</v>
+      </c>
+      <c r="I18" s="6" t="n">
+        <v>51.53</v>
+      </c>
       <c r="J18" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1131,12 +1235,20 @@
         <v>0.504</v>
       </c>
       <c r="E19" s="8" t="n">
-        <v>3.668</v>
-      </c>
-      <c r="F19" s="8" t="n"/>
-      <c r="G19" s="8" t="n"/>
-      <c r="H19" s="8" t="n"/>
-      <c r="I19" s="8" t="n"/>
+        <v>0.76415</v>
+      </c>
+      <c r="F19" s="8" t="n">
+        <v>53.415</v>
+      </c>
+      <c r="G19" s="8" t="n">
+        <v>47.927</v>
+      </c>
+      <c r="H19" s="8" t="n">
+        <v>54.982</v>
+      </c>
+      <c r="I19" s="8" t="n">
+        <v>51.916</v>
+      </c>
       <c r="J19" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1174,12 +1286,20 @@
         <v>0.171</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>2.919</v>
-      </c>
-      <c r="F20" s="6" t="n"/>
-      <c r="G20" s="6" t="n"/>
-      <c r="H20" s="6" t="n"/>
-      <c r="I20" s="6" t="n"/>
+        <v>-1.641393</v>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>53.622</v>
+      </c>
+      <c r="G20" s="6" t="n">
+        <v>48.044</v>
+      </c>
+      <c r="H20" s="6" t="n">
+        <v>55.745</v>
+      </c>
+      <c r="I20" s="6" t="n">
+        <v>51.779</v>
+      </c>
       <c r="J20" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1217,12 +1337,20 @@
         <v>0.02</v>
       </c>
       <c r="E21" s="8" t="n">
-        <v>2.936</v>
-      </c>
-      <c r="F21" s="8" t="n"/>
-      <c r="G21" s="8" t="n"/>
-      <c r="H21" s="8" t="n"/>
-      <c r="I21" s="8" t="n"/>
+        <v>0.033758</v>
+      </c>
+      <c r="F21" s="8" t="n">
+        <v>53.358</v>
+      </c>
+      <c r="G21" s="8" t="n">
+        <v>48.506</v>
+      </c>
+      <c r="H21" s="8" t="n">
+        <v>56.078</v>
+      </c>
+      <c r="I21" s="8" t="n">
+        <v>51.682</v>
+      </c>
       <c r="J21" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1260,12 +1388,20 @@
         <v>-1.413</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>2.378</v>
-      </c>
-      <c r="F22" s="6" t="n"/>
-      <c r="G22" s="6" t="n"/>
-      <c r="H22" s="6" t="n"/>
-      <c r="I22" s="6" t="n"/>
+        <v>-1.036342</v>
+      </c>
+      <c r="F22" s="6" t="n">
+        <v>53.181</v>
+      </c>
+      <c r="G22" s="6" t="n">
+        <v>48.395</v>
+      </c>
+      <c r="H22" s="6" t="n">
+        <v>53.562</v>
+      </c>
+      <c r="I22" s="6" t="n">
+        <v>49.999</v>
+      </c>
       <c r="J22" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1303,12 +1439,20 @@
         <v>-0.892</v>
       </c>
       <c r="E23" s="8" t="n">
-        <v>2.264</v>
-      </c>
-      <c r="F23" s="8" t="n"/>
-      <c r="G23" s="8" t="n"/>
-      <c r="H23" s="8" t="n"/>
-      <c r="I23" s="8" t="n"/>
+        <v>-0.158137</v>
+      </c>
+      <c r="F23" s="8" t="n">
+        <v>51.709</v>
+      </c>
+      <c r="G23" s="8" t="n">
+        <v>47.852</v>
+      </c>
+      <c r="H23" s="8" t="n">
+        <v>53.495</v>
+      </c>
+      <c r="I23" s="8" t="n">
+        <v>48.883</v>
+      </c>
       <c r="J23" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1346,12 +1490,20 @@
         <v>-0.993</v>
       </c>
       <c r="E24" s="6" t="n">
-        <v>-3.083</v>
-      </c>
-      <c r="F24" s="6" t="n"/>
-      <c r="G24" s="6" t="n"/>
-      <c r="H24" s="6" t="n"/>
-      <c r="I24" s="6" t="n"/>
+        <v>-10.562397</v>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>50.653</v>
+      </c>
+      <c r="G24" s="6" t="n">
+        <v>47.003</v>
+      </c>
+      <c r="H24" s="6" t="n">
+        <v>51.916</v>
+      </c>
+      <c r="I24" s="6" t="n">
+        <v>48.188</v>
+      </c>
       <c r="J24" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1389,12 +1541,20 @@
         <v>-0.524</v>
       </c>
       <c r="E25" s="8" t="n">
-        <v>-4.261</v>
-      </c>
-      <c r="F25" s="8" t="n"/>
-      <c r="G25" s="8" t="n"/>
-      <c r="H25" s="8" t="n"/>
-      <c r="I25" s="8" t="n"/>
+        <v>-2.141653</v>
+      </c>
+      <c r="F25" s="8" t="n">
+        <v>50.317</v>
+      </c>
+      <c r="G25" s="8" t="n">
+        <v>46.905</v>
+      </c>
+      <c r="H25" s="8" t="n">
+        <v>51.029</v>
+      </c>
+      <c r="I25" s="8" t="n">
+        <v>47.677</v>
+      </c>
       <c r="J25" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1432,12 +1592,20 @@
         <v>0.842</v>
       </c>
       <c r="E26" s="6" t="n">
-        <v>-2.278</v>
-      </c>
-      <c r="F26" s="6" t="n"/>
-      <c r="G26" s="6" t="n"/>
-      <c r="H26" s="6" t="n"/>
-      <c r="I26" s="6" t="n"/>
+        <v>3.63273</v>
+      </c>
+      <c r="F26" s="6" t="n">
+        <v>51.014</v>
+      </c>
+      <c r="G26" s="6" t="n">
+        <v>47.828</v>
+      </c>
+      <c r="H26" s="6" t="n">
+        <v>52.502</v>
+      </c>
+      <c r="I26" s="6" t="n">
+        <v>48.248</v>
+      </c>
       <c r="J26" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1475,12 +1643,20 @@
         <v>-1.299</v>
       </c>
       <c r="E27" s="8" t="n">
-        <v>-3.081</v>
-      </c>
-      <c r="F27" s="8" t="n"/>
-      <c r="G27" s="8" t="n"/>
-      <c r="H27" s="8" t="n"/>
-      <c r="I27" s="8" t="n"/>
+        <v>-1.598997</v>
+      </c>
+      <c r="F27" s="8" t="n">
+        <v>50.226</v>
+      </c>
+      <c r="G27" s="8" t="n">
+        <v>47.166</v>
+      </c>
+      <c r="H27" s="8" t="n">
+        <v>51.411</v>
+      </c>
+      <c r="I27" s="8" t="n">
+        <v>46.48</v>
+      </c>
       <c r="J27" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1518,12 +1694,20 @@
         <v>-0.759</v>
       </c>
       <c r="E28" s="6" t="n">
-        <v>-2.376</v>
-      </c>
-      <c r="F28" s="6" t="n"/>
-      <c r="G28" s="6" t="n"/>
-      <c r="H28" s="6" t="n"/>
-      <c r="I28" s="6" t="n"/>
+        <v>1.232329</v>
+      </c>
+      <c r="F28" s="6" t="n">
+        <v>49.526</v>
+      </c>
+      <c r="G28" s="6" t="n">
+        <v>45.704</v>
+      </c>
+      <c r="H28" s="6" t="n">
+        <v>49.687</v>
+      </c>
+      <c r="I28" s="6" t="n">
+        <v>46.328</v>
+      </c>
       <c r="J28" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1561,12 +1745,20 @@
         <v>0.424</v>
       </c>
       <c r="E29" s="8" t="n">
-        <v>-2.507</v>
-      </c>
-      <c r="F29" s="8" t="n"/>
-      <c r="G29" s="8" t="n"/>
-      <c r="H29" s="8" t="n"/>
-      <c r="I29" s="8" t="n"/>
+        <v>-0.206614</v>
+      </c>
+      <c r="F29" s="8" t="n">
+        <v>49.079</v>
+      </c>
+      <c r="G29" s="8" t="n">
+        <v>47.312</v>
+      </c>
+      <c r="H29" s="8" t="n">
+        <v>51.16</v>
+      </c>
+      <c r="I29" s="8" t="n">
+        <v>46.377</v>
+      </c>
       <c r="J29" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1604,12 +1796,20 @@
         <v>-0.9399999999999999</v>
       </c>
       <c r="E30" s="6" t="n">
-        <v>-4.859</v>
-      </c>
-      <c r="F30" s="6" t="n"/>
-      <c r="G30" s="6" t="n"/>
-      <c r="H30" s="6" t="n"/>
-      <c r="I30" s="6" t="n"/>
+        <v>-4.382062</v>
+      </c>
+      <c r="F30" s="6" t="n">
+        <v>48.445</v>
+      </c>
+      <c r="G30" s="6" t="n">
+        <v>45.917</v>
+      </c>
+      <c r="H30" s="6" t="n">
+        <v>51.535</v>
+      </c>
+      <c r="I30" s="6" t="n">
+        <v>44.718</v>
+      </c>
       <c r="J30" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1647,12 +1847,20 @@
         <v>1.071</v>
       </c>
       <c r="E31" s="8" t="n">
-        <v>-4.292</v>
-      </c>
-      <c r="F31" s="8" t="n"/>
-      <c r="G31" s="8" t="n"/>
-      <c r="H31" s="8" t="n"/>
-      <c r="I31" s="8" t="n"/>
+        <v>1.167722</v>
+      </c>
+      <c r="F31" s="8" t="n">
+        <v>47.757</v>
+      </c>
+      <c r="G31" s="8" t="n">
+        <v>44.829</v>
+      </c>
+      <c r="H31" s="8" t="n">
+        <v>51.263</v>
+      </c>
+      <c r="I31" s="8" t="n">
+        <v>47.721</v>
+      </c>
       <c r="J31" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1690,12 +1898,20 @@
         <v>-4.384</v>
       </c>
       <c r="E32" s="6" t="n">
-        <v>-8.847</v>
-      </c>
-      <c r="F32" s="6" t="n"/>
-      <c r="G32" s="6" t="n"/>
-      <c r="H32" s="6" t="n"/>
-      <c r="I32" s="6" t="n"/>
+        <v>-8.607958</v>
+      </c>
+      <c r="F32" s="6" t="n">
+        <v>44.397</v>
+      </c>
+      <c r="G32" s="6" t="n">
+        <v>43.45</v>
+      </c>
+      <c r="H32" s="6" t="n">
+        <v>46.475</v>
+      </c>
+      <c r="I32" s="6" t="n">
+        <v>42.463</v>
+      </c>
       <c r="J32" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1733,12 +1949,20 @@
         <v>-8.247</v>
       </c>
       <c r="E33" s="8" t="n">
-        <v>-17.114</v>
-      </c>
-      <c r="F33" s="8" t="n"/>
-      <c r="G33" s="8" t="n"/>
-      <c r="H33" s="8" t="n"/>
-      <c r="I33" s="8" t="n"/>
+        <v>-15.658555</v>
+      </c>
+      <c r="F33" s="8" t="n">
+        <v>36.578</v>
+      </c>
+      <c r="G33" s="8" t="n">
+        <v>37.197</v>
+      </c>
+      <c r="H33" s="8" t="n">
+        <v>39.131</v>
+      </c>
+      <c r="I33" s="8" t="n">
+        <v>33.157</v>
+      </c>
       <c r="J33" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1776,12 +2000,20 @@
         <v>-1.76</v>
       </c>
       <c r="E34" s="6" t="n">
-        <v>-17.461</v>
-      </c>
-      <c r="F34" s="6" t="n"/>
-      <c r="G34" s="6" t="n"/>
-      <c r="H34" s="6" t="n"/>
-      <c r="I34" s="6" t="n"/>
+        <v>-1.567765</v>
+      </c>
+      <c r="F34" s="6" t="n">
+        <v>34.285</v>
+      </c>
+      <c r="G34" s="6" t="n">
+        <v>34.752</v>
+      </c>
+      <c r="H34" s="6" t="n">
+        <v>37.898</v>
+      </c>
+      <c r="I34" s="6" t="n">
+        <v>31.511</v>
+      </c>
       <c r="J34" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1819,12 +2051,20 @@
         <v>2.509</v>
       </c>
       <c r="E35" s="8" t="n">
-        <v>-14.06</v>
-      </c>
-      <c r="F35" s="8" t="n"/>
-      <c r="G35" s="8" t="n"/>
-      <c r="H35" s="8" t="n"/>
-      <c r="I35" s="8" t="n"/>
+        <v>6.137927</v>
+      </c>
+      <c r="F35" s="8" t="n">
+        <v>37.29</v>
+      </c>
+      <c r="G35" s="8" t="n">
+        <v>35.051</v>
+      </c>
+      <c r="H35" s="8" t="n">
+        <v>38.35</v>
+      </c>
+      <c r="I35" s="8" t="n">
+        <v>35.287</v>
+      </c>
       <c r="J35" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1862,12 +2102,20 @@
         <v>2.131</v>
       </c>
       <c r="E36" s="6" t="n">
-        <v>-10.936</v>
-      </c>
-      <c r="F36" s="6" t="n"/>
-      <c r="G36" s="6" t="n"/>
-      <c r="H36" s="6" t="n"/>
-      <c r="I36" s="6" t="n"/>
+        <v>5.755039</v>
+      </c>
+      <c r="F36" s="6" t="n">
+        <v>39.015</v>
+      </c>
+      <c r="G36" s="6" t="n">
+        <v>39.375</v>
+      </c>
+      <c r="H36" s="6" t="n">
+        <v>41.349</v>
+      </c>
+      <c r="I36" s="6" t="n">
+        <v>36.719</v>
+      </c>
       <c r="J36" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1905,12 +2153,20 @@
         <v>-0.617</v>
       </c>
       <c r="E37" s="8" t="n">
-        <v>-11.029</v>
-      </c>
-      <c r="F37" s="8" t="n"/>
-      <c r="G37" s="8" t="n"/>
-      <c r="H37" s="8" t="n"/>
-      <c r="I37" s="8" t="n"/>
+        <v>-0.426587</v>
+      </c>
+      <c r="F37" s="8" t="n">
+        <v>38.629</v>
+      </c>
+      <c r="G37" s="8" t="n">
+        <v>38.464</v>
+      </c>
+      <c r="H37" s="8" t="n">
+        <v>42.073</v>
+      </c>
+      <c r="I37" s="8" t="n">
+        <v>35.371</v>
+      </c>
       <c r="J37" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1948,12 +2204,20 @@
         <v>0.898</v>
       </c>
       <c r="E38" s="6" t="n">
-        <v>-10.973</v>
-      </c>
-      <c r="F38" s="6" t="n"/>
-      <c r="G38" s="6" t="n"/>
-      <c r="H38" s="6" t="n"/>
-      <c r="I38" s="6" t="n"/>
+        <v>0.493442</v>
+      </c>
+      <c r="F38" s="6" t="n">
+        <v>41.042</v>
+      </c>
+      <c r="G38" s="6" t="n">
+        <v>40.081</v>
+      </c>
+      <c r="H38" s="6" t="n">
+        <v>41.799</v>
+      </c>
+      <c r="I38" s="6" t="n">
+        <v>36.025</v>
+      </c>
       <c r="J38" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1991,12 +2255,20 @@
         <v>1.245</v>
       </c>
       <c r="E39" s="8" t="n">
-        <v>-8.429</v>
-      </c>
-      <c r="F39" s="8" t="n"/>
-      <c r="G39" s="8" t="n"/>
-      <c r="H39" s="8" t="n"/>
-      <c r="I39" s="8" t="n"/>
+        <v>4.655618</v>
+      </c>
+      <c r="F39" s="8" t="n">
+        <v>41.767</v>
+      </c>
+      <c r="G39" s="8" t="n">
+        <v>40.883</v>
+      </c>
+      <c r="H39" s="8" t="n">
+        <v>42.921</v>
+      </c>
+      <c r="I39" s="8" t="n">
+        <v>37.661</v>
+      </c>
       <c r="J39" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2034,12 +2306,20 @@
         <v>-0.164</v>
       </c>
       <c r="E40" s="6" t="n">
-        <v>-7.834</v>
-      </c>
-      <c r="F40" s="6" t="n"/>
-      <c r="G40" s="6" t="n"/>
-      <c r="H40" s="6" t="n"/>
-      <c r="I40" s="6" t="n"/>
+        <v>0.970079</v>
+      </c>
+      <c r="F40" s="6" t="n">
+        <v>42.139</v>
+      </c>
+      <c r="G40" s="6" t="n">
+        <v>41.367</v>
+      </c>
+      <c r="H40" s="6" t="n">
+        <v>43.59</v>
+      </c>
+      <c r="I40" s="6" t="n">
+        <v>36.695</v>
+      </c>
       <c r="J40" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2077,12 +2357,20 @@
         <v>1.172</v>
       </c>
       <c r="E41" s="8" t="n">
-        <v>-7.086</v>
-      </c>
-      <c r="F41" s="8" t="n"/>
-      <c r="G41" s="8" t="n"/>
-      <c r="H41" s="8" t="n"/>
-      <c r="I41" s="8" t="n"/>
+        <v>1.697639</v>
+      </c>
+      <c r="F41" s="8" t="n">
+        <v>42.998</v>
+      </c>
+      <c r="G41" s="8" t="n">
+        <v>41.97</v>
+      </c>
+      <c r="H41" s="8" t="n">
+        <v>44.841</v>
+      </c>
+      <c r="I41" s="8" t="n">
+        <v>38.086</v>
+      </c>
       <c r="J41" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2120,12 +2408,20 @@
         <v>-0.108</v>
       </c>
       <c r="E42" s="6" t="n">
-        <v>-6.254</v>
-      </c>
-      <c r="F42" s="6" t="n"/>
-      <c r="G42" s="6" t="n"/>
-      <c r="H42" s="6" t="n"/>
-      <c r="I42" s="6" t="n"/>
+        <v>1.469067</v>
+      </c>
+      <c r="F42" s="6" t="n">
+        <v>43.668</v>
+      </c>
+      <c r="G42" s="6" t="n">
+        <v>42.347</v>
+      </c>
+      <c r="H42" s="6" t="n">
+        <v>45.468</v>
+      </c>
+      <c r="I42" s="6" t="n">
+        <v>37.146</v>
+      </c>
       <c r="J42" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2163,12 +2459,20 @@
         <v>1.201</v>
       </c>
       <c r="E43" s="8" t="n">
-        <v>-6.124</v>
-      </c>
-      <c r="F43" s="8" t="n"/>
-      <c r="G43" s="8" t="n"/>
-      <c r="H43" s="8" t="n"/>
-      <c r="I43" s="8" t="n"/>
+        <v>0.562936</v>
+      </c>
+      <c r="F43" s="8" t="n">
+        <v>44.653</v>
+      </c>
+      <c r="G43" s="8" t="n">
+        <v>43.085</v>
+      </c>
+      <c r="H43" s="8" t="n">
+        <v>45.675</v>
+      </c>
+      <c r="I43" s="8" t="n">
+        <v>39.049</v>
+      </c>
       <c r="J43" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2206,12 +2510,20 @@
         <v>2.961</v>
       </c>
       <c r="E44" s="6" t="n">
-        <v>1.221</v>
-      </c>
-      <c r="F44" s="6" t="n"/>
-      <c r="G44" s="6" t="n"/>
-      <c r="H44" s="6" t="n"/>
-      <c r="I44" s="6" t="n"/>
+        <v>15.46233</v>
+      </c>
+      <c r="F44" s="6" t="n">
+        <v>46.021</v>
+      </c>
+      <c r="G44" s="6" t="n">
+        <v>43.884</v>
+      </c>
+      <c r="H44" s="6" t="n">
+        <v>49.164</v>
+      </c>
+      <c r="I44" s="6" t="n">
+        <v>42.91</v>
+      </c>
       <c r="J44" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2249,12 +2561,20 @@
         <v>2.18</v>
       </c>
       <c r="E45" s="8" t="n">
-        <v>11.648</v>
-      </c>
-      <c r="F45" s="8" t="n"/>
-      <c r="G45" s="8" t="n"/>
-      <c r="H45" s="8" t="n"/>
-      <c r="I45" s="8" t="n"/>
+        <v>29.883172</v>
+      </c>
+      <c r="F45" s="8" t="n">
+        <v>48.687</v>
+      </c>
+      <c r="G45" s="8" t="n">
+        <v>44.61</v>
+      </c>
+      <c r="H45" s="8" t="n">
+        <v>51.056</v>
+      </c>
+      <c r="I45" s="8" t="n">
+        <v>45.307</v>
+      </c>
       <c r="J45" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2292,12 +2612,20 @@
         <v>1.762</v>
       </c>
       <c r="E46" s="6" t="n">
-        <v>15.17</v>
-      </c>
-      <c r="F46" s="6" t="n"/>
-      <c r="G46" s="6" t="n"/>
-      <c r="H46" s="6" t="n"/>
-      <c r="I46" s="6" t="n"/>
+        <v>12.085213</v>
+      </c>
+      <c r="F46" s="6" t="n">
+        <v>49.692</v>
+      </c>
+      <c r="G46" s="6" t="n">
+        <v>45.781</v>
+      </c>
+      <c r="H46" s="6" t="n">
+        <v>52.246</v>
+      </c>
+      <c r="I46" s="6" t="n">
+        <v>47.827</v>
+      </c>
       <c r="J46" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2335,12 +2663,20 @@
         <v>2.173</v>
       </c>
       <c r="E47" s="8" t="n">
-        <v>14.834</v>
-      </c>
-      <c r="F47" s="8" t="n"/>
-      <c r="G47" s="8" t="n"/>
-      <c r="H47" s="8" t="n"/>
-      <c r="I47" s="8" t="n"/>
+        <v>-4.006589</v>
+      </c>
+      <c r="F47" s="8" t="n">
+        <v>51.361</v>
+      </c>
+      <c r="G47" s="8" t="n">
+        <v>47.838</v>
+      </c>
+      <c r="H47" s="8" t="n">
+        <v>54.196</v>
+      </c>
+      <c r="I47" s="8" t="n">
+        <v>50.371</v>
+      </c>
       <c r="J47" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2378,12 +2714,20 @@
         <v>-0.083</v>
       </c>
       <c r="E48" s="6" t="n">
-        <v>12.62</v>
-      </c>
-      <c r="F48" s="6" t="n"/>
-      <c r="G48" s="6" t="n"/>
-      <c r="H48" s="6" t="n"/>
-      <c r="I48" s="6" t="n"/>
+        <v>-7.997474</v>
+      </c>
+      <c r="F48" s="6" t="n">
+        <v>51.881</v>
+      </c>
+      <c r="G48" s="6" t="n">
+        <v>49.015</v>
+      </c>
+      <c r="H48" s="6" t="n">
+        <v>54.558</v>
+      </c>
+      <c r="I48" s="6" t="n">
+        <v>49.528</v>
+      </c>
       <c r="J48" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2421,12 +2765,20 @@
         <v>-1.394</v>
       </c>
       <c r="E49" s="8" t="n">
-        <v>11.843</v>
-      </c>
-      <c r="F49" s="8" t="n"/>
-      <c r="G49" s="8" t="n"/>
-      <c r="H49" s="8" t="n"/>
-      <c r="I49" s="8" t="n"/>
+        <v>-1.51613</v>
+      </c>
+      <c r="F49" s="8" t="n">
+        <v>50.804</v>
+      </c>
+      <c r="G49" s="8" t="n">
+        <v>46.393</v>
+      </c>
+      <c r="H49" s="8" t="n">
+        <v>53.506</v>
+      </c>
+      <c r="I49" s="8" t="n">
+        <v>48.062</v>
+      </c>
       <c r="J49" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2464,12 +2816,20 @@
         <v>1.429</v>
       </c>
       <c r="E50" s="6" t="n">
-        <v>12.374</v>
-      </c>
-      <c r="F50" s="6" t="n"/>
-      <c r="G50" s="6" t="n"/>
-      <c r="H50" s="6" t="n"/>
-      <c r="I50" s="6" t="n"/>
+        <v>0.645431</v>
+      </c>
+      <c r="F50" s="6" t="n">
+        <v>51.636</v>
+      </c>
+      <c r="G50" s="6" t="n">
+        <v>48.16</v>
+      </c>
+      <c r="H50" s="6" t="n">
+        <v>54.933</v>
+      </c>
+      <c r="I50" s="6" t="n">
+        <v>49.698</v>
+      </c>
       <c r="J50" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2507,12 +2867,20 @@
         <v>0.828</v>
       </c>
       <c r="E51" s="8" t="n">
-        <v>11.957</v>
-      </c>
-      <c r="F51" s="8" t="n"/>
-      <c r="G51" s="8" t="n"/>
-      <c r="H51" s="8" t="n"/>
-      <c r="I51" s="8" t="n"/>
+        <v>-2.031242</v>
+      </c>
+      <c r="F51" s="8" t="n">
+        <v>52.061</v>
+      </c>
+      <c r="G51" s="8" t="n">
+        <v>48.992</v>
+      </c>
+      <c r="H51" s="8" t="n">
+        <v>54.825</v>
+      </c>
+      <c r="I51" s="8" t="n">
+        <v>51.189</v>
+      </c>
       <c r="J51" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2550,12 +2918,20 @@
         <v>1.446</v>
       </c>
       <c r="E52" s="6" t="n">
-        <v>13.567</v>
-      </c>
-      <c r="F52" s="6" t="n"/>
-      <c r="G52" s="6" t="n"/>
-      <c r="H52" s="6" t="n"/>
-      <c r="I52" s="6" t="n"/>
+        <v>4.157543</v>
+      </c>
+      <c r="F52" s="6" t="n">
+        <v>52.722</v>
+      </c>
+      <c r="G52" s="6" t="n">
+        <v>50.477</v>
+      </c>
+      <c r="H52" s="6" t="n">
+        <v>56.56</v>
+      </c>
+      <c r="I52" s="6" t="n">
+        <v>52.84</v>
+      </c>
       <c r="J52" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2593,12 +2969,20 @@
         <v>1.434</v>
       </c>
       <c r="E53" s="8" t="n">
-        <v>13.829</v>
-      </c>
-      <c r="F53" s="8" t="n"/>
-      <c r="G53" s="8" t="n"/>
-      <c r="H53" s="8" t="n"/>
-      <c r="I53" s="8" t="n"/>
+        <v>-0.332301</v>
+      </c>
+      <c r="F53" s="8" t="n">
+        <v>52.703</v>
+      </c>
+      <c r="G53" s="8" t="n">
+        <v>50.895</v>
+      </c>
+      <c r="H53" s="8" t="n">
+        <v>57.434</v>
+      </c>
+      <c r="I53" s="8" t="n">
+        <v>55.435</v>
+      </c>
       <c r="J53" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2636,12 +3020,20 @@
         <v>-3.44</v>
       </c>
       <c r="E54" s="6" t="n">
-        <v>10.497</v>
-      </c>
-      <c r="F54" s="6" t="n"/>
-      <c r="G54" s="6" t="n"/>
-      <c r="H54" s="6" t="n"/>
-      <c r="I54" s="6" t="n"/>
+        <v>-8.044813</v>
+      </c>
+      <c r="F54" s="6" t="n">
+        <v>51.167</v>
+      </c>
+      <c r="G54" s="6" t="n">
+        <v>50.177</v>
+      </c>
+      <c r="H54" s="6" t="n">
+        <v>55.999</v>
+      </c>
+      <c r="I54" s="6" t="n">
+        <v>49.546</v>
+      </c>
       <c r="J54" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2679,12 +3071,20 @@
         <v>0.579</v>
       </c>
       <c r="E55" s="8" t="n">
-        <v>9.875</v>
-      </c>
-      <c r="F55" s="8" t="n"/>
-      <c r="G55" s="8" t="n"/>
-      <c r="H55" s="8" t="n"/>
-      <c r="I55" s="8" t="n"/>
+        <v>-2.204901</v>
+      </c>
+      <c r="F55" s="8" t="n">
+        <v>52.914</v>
+      </c>
+      <c r="G55" s="8" t="n">
+        <v>51.157</v>
+      </c>
+      <c r="H55" s="8" t="n">
+        <v>54.711</v>
+      </c>
+      <c r="I55" s="8" t="n">
+        <v>50.459</v>
+      </c>
       <c r="J55" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2722,12 +3122,20 @@
         <v>-0.08400000000000001</v>
       </c>
       <c r="E56" s="6" t="n">
-        <v>6.83</v>
-      </c>
-      <c r="F56" s="6" t="n"/>
-      <c r="G56" s="6" t="n"/>
-      <c r="H56" s="6" t="n"/>
-      <c r="I56" s="6" t="n"/>
+        <v>-8.284058999999999</v>
+      </c>
+      <c r="F56" s="6" t="n">
+        <v>51.825</v>
+      </c>
+      <c r="G56" s="6" t="n">
+        <v>51.798</v>
+      </c>
+      <c r="H56" s="6" t="n">
+        <v>53.956</v>
+      </c>
+      <c r="I56" s="6" t="n">
+        <v>51.032</v>
+      </c>
       <c r="J56" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2765,12 +3173,20 @@
         <v>1.585</v>
       </c>
       <c r="E57" s="8" t="n">
-        <v>6.235</v>
-      </c>
-      <c r="F57" s="8" t="n"/>
-      <c r="G57" s="8" t="n"/>
-      <c r="H57" s="8" t="n"/>
-      <c r="I57" s="8" t="n"/>
+        <v>-1.955139</v>
+      </c>
+      <c r="F57" s="8" t="n">
+        <v>52.608</v>
+      </c>
+      <c r="G57" s="8" t="n">
+        <v>51.088</v>
+      </c>
+      <c r="H57" s="8" t="n">
+        <v>55.453</v>
+      </c>
+      <c r="I57" s="8" t="n">
+        <v>53.496</v>
+      </c>
       <c r="J57" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2808,12 +3224,20 @@
         <v>-0.602</v>
       </c>
       <c r="E58" s="6" t="n">
-        <v>3.871</v>
-      </c>
-      <c r="F58" s="6" t="n"/>
-      <c r="G58" s="6" t="n"/>
-      <c r="H58" s="6" t="n"/>
-      <c r="I58" s="6" t="n"/>
+        <v>-5.290859</v>
+      </c>
+      <c r="F58" s="6" t="n">
+        <v>52.497</v>
+      </c>
+      <c r="G58" s="6" t="n">
+        <v>49.749</v>
+      </c>
+      <c r="H58" s="6" t="n">
+        <v>54.683</v>
+      </c>
+      <c r="I58" s="6" t="n">
+        <v>52.901</v>
+      </c>
       <c r="J58" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2851,12 +3275,20 @@
         <v>-1.432</v>
       </c>
       <c r="E59" s="8" t="n">
-        <v>0.266</v>
-      </c>
-      <c r="F59" s="8" t="n"/>
-      <c r="G59" s="8" t="n"/>
-      <c r="H59" s="8" t="n"/>
-      <c r="I59" s="8" t="n"/>
+        <v>-7.369635</v>
+      </c>
+      <c r="F59" s="8" t="n">
+        <v>52.168</v>
+      </c>
+      <c r="G59" s="8" t="n">
+        <v>51.099</v>
+      </c>
+      <c r="H59" s="8" t="n">
+        <v>55.841</v>
+      </c>
+      <c r="I59" s="8" t="n">
+        <v>49.078</v>
+      </c>
       <c r="J59" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2894,12 +3326,20 @@
         <v>-1.056</v>
       </c>
       <c r="E60" s="6" t="n">
-        <v>-0.707</v>
-      </c>
-      <c r="F60" s="6" t="n"/>
-      <c r="G60" s="6" t="n"/>
-      <c r="H60" s="6" t="n"/>
-      <c r="I60" s="6" t="n"/>
+        <v>-1.901034</v>
+      </c>
+      <c r="F60" s="6" t="n">
+        <v>51.219</v>
+      </c>
+      <c r="G60" s="6" t="n">
+        <v>49.85</v>
+      </c>
+      <c r="H60" s="6" t="n">
+        <v>55.175</v>
+      </c>
+      <c r="I60" s="6" t="n">
+        <v>47.815</v>
+      </c>
       <c r="J60" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2937,12 +3377,20 @@
         <v>-2.001</v>
       </c>
       <c r="E61" s="8" t="n">
-        <v>-1.314</v>
-      </c>
-      <c r="F61" s="8" t="n"/>
-      <c r="G61" s="8" t="n"/>
-      <c r="H61" s="8" t="n"/>
-      <c r="I61" s="8" t="n"/>
+        <v>-1.258418</v>
+      </c>
+      <c r="F61" s="8" t="n">
+        <v>51.297</v>
+      </c>
+      <c r="G61" s="8" t="n">
+        <v>48.541</v>
+      </c>
+      <c r="H61" s="8" t="n">
+        <v>53.822</v>
+      </c>
+      <c r="I61" s="8" t="n">
+        <v>44.386</v>
+      </c>
       <c r="J61" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2980,12 +3428,20 @@
         <v>-0.488</v>
       </c>
       <c r="E62" s="6" t="n">
-        <v>-3.231</v>
-      </c>
-      <c r="F62" s="6" t="n"/>
-      <c r="G62" s="6" t="n"/>
-      <c r="H62" s="6" t="n"/>
-      <c r="I62" s="6" t="n"/>
+        <v>-3.670806</v>
+      </c>
+      <c r="F62" s="6" t="n">
+        <v>50.889</v>
+      </c>
+      <c r="G62" s="6" t="n">
+        <v>50.977</v>
+      </c>
+      <c r="H62" s="6" t="n">
+        <v>53.657</v>
+      </c>
+      <c r="I62" s="6" t="n">
+        <v>43.105</v>
+      </c>
       <c r="J62" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3023,12 +3479,20 @@
         <v>1.884</v>
       </c>
       <c r="E63" s="8" t="n">
-        <v>-2.175</v>
-      </c>
-      <c r="F63" s="8" t="n"/>
-      <c r="G63" s="8" t="n"/>
-      <c r="H63" s="8" t="n"/>
-      <c r="I63" s="8" t="n"/>
+        <v>2.13032</v>
+      </c>
+      <c r="F63" s="8" t="n">
+        <v>50.728</v>
+      </c>
+      <c r="G63" s="8" t="n">
+        <v>51.357</v>
+      </c>
+      <c r="H63" s="8" t="n">
+        <v>52.789</v>
+      </c>
+      <c r="I63" s="8" t="n">
+        <v>47.638</v>
+      </c>
       <c r="J63" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3066,12 +3530,20 @@
         <v>-0.245</v>
       </c>
       <c r="E64" s="6" t="n">
-        <v>-3.866</v>
-      </c>
-      <c r="F64" s="6" t="n"/>
-      <c r="G64" s="6" t="n"/>
-      <c r="H64" s="6" t="n"/>
-      <c r="I64" s="6" t="n"/>
+        <v>-3.049515</v>
+      </c>
+      <c r="F64" s="6" t="n">
+        <v>50.111</v>
+      </c>
+      <c r="G64" s="6" t="n">
+        <v>50.505</v>
+      </c>
+      <c r="H64" s="6" t="n">
+        <v>52.743</v>
+      </c>
+      <c r="I64" s="6" t="n">
+        <v>47.585</v>
+      </c>
       <c r="J64" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3109,12 +3581,20 @@
         <v>-2.201</v>
       </c>
       <c r="E65" s="8" t="n">
-        <v>-7.501</v>
-      </c>
-      <c r="F65" s="8" t="n"/>
-      <c r="G65" s="8" t="n"/>
-      <c r="H65" s="8" t="n"/>
-      <c r="I65" s="8" t="n"/>
+        <v>-6.431919</v>
+      </c>
+      <c r="F65" s="8" t="n">
+        <v>50.36</v>
+      </c>
+      <c r="G65" s="8" t="n">
+        <v>48.227</v>
+      </c>
+      <c r="H65" s="8" t="n">
+        <v>52.498</v>
+      </c>
+      <c r="I65" s="8" t="n">
+        <v>43.275</v>
+      </c>
       <c r="J65" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3152,12 +3632,20 @@
         <v>1.148</v>
       </c>
       <c r="E66" s="6" t="n">
-        <v>-2.913</v>
-      </c>
-      <c r="F66" s="6" t="n"/>
-      <c r="G66" s="6" t="n"/>
-      <c r="H66" s="6" t="n"/>
-      <c r="I66" s="6" t="n"/>
+        <v>8.001899999999999</v>
+      </c>
+      <c r="F66" s="6" t="n">
+        <v>50.966</v>
+      </c>
+      <c r="G66" s="6" t="n">
+        <v>53.3</v>
+      </c>
+      <c r="H66" s="6" t="n">
+        <v>53.615</v>
+      </c>
+      <c r="I66" s="6" t="n">
+        <v>43.894</v>
+      </c>
       <c r="J66" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3195,12 +3683,20 @@
         <v>3.225</v>
       </c>
       <c r="E67" s="8" t="n">
-        <v>-0.267</v>
-      </c>
-      <c r="F67" s="8" t="n"/>
-      <c r="G67" s="8" t="n"/>
-      <c r="H67" s="8" t="n"/>
-      <c r="I67" s="8" t="n"/>
+        <v>5.14733</v>
+      </c>
+      <c r="F67" s="8" t="n">
+        <v>53.506</v>
+      </c>
+      <c r="G67" s="8" t="n">
+        <v>52.528</v>
+      </c>
+      <c r="H67" s="8" t="n">
+        <v>54.346</v>
+      </c>
+      <c r="I67" s="8" t="n">
+        <v>49.515</v>
+      </c>
       <c r="J67" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3238,12 +3734,20 @@
         <v>1.836</v>
       </c>
       <c r="E68" s="6" t="n">
-        <v>1.653</v>
-      </c>
-      <c r="F68" s="6" t="n"/>
-      <c r="G68" s="6" t="n"/>
-      <c r="H68" s="6" t="n"/>
-      <c r="I68" s="6" t="n"/>
+        <v>3.694463</v>
+      </c>
+      <c r="F68" s="6" t="n">
+        <v>53.419</v>
+      </c>
+      <c r="G68" s="6" t="n">
+        <v>51.35</v>
+      </c>
+      <c r="H68" s="6" t="n">
+        <v>53.577</v>
+      </c>
+      <c r="I68" s="6" t="n">
+        <v>54.174</v>
+      </c>
       <c r="J68" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3281,12 +3785,20 @@
         <v>1.165</v>
       </c>
       <c r="E69" s="8" t="n">
-        <v>1.233</v>
-      </c>
-      <c r="F69" s="8" t="n"/>
-      <c r="G69" s="8" t="n"/>
-      <c r="H69" s="8" t="n"/>
-      <c r="I69" s="8" t="n"/>
+        <v>-0.878594</v>
+      </c>
+      <c r="F69" s="8" t="n">
+        <v>53.44</v>
+      </c>
+      <c r="G69" s="8" t="n">
+        <v>54.818</v>
+      </c>
+      <c r="H69" s="8" t="n">
+        <v>55.548</v>
+      </c>
+      <c r="I69" s="8" t="n">
+        <v>54.989</v>
+      </c>
       <c r="J69" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3324,12 +3836,20 @@
         <v>0.904</v>
       </c>
       <c r="E70" s="6" t="n">
-        <v>2.739</v>
-      </c>
-      <c r="F70" s="6" t="n"/>
-      <c r="G70" s="6" t="n"/>
-      <c r="H70" s="6" t="n"/>
-      <c r="I70" s="6" t="n"/>
+        <v>2.870862</v>
+      </c>
+      <c r="F70" s="6" t="n">
+        <v>53.61</v>
+      </c>
+      <c r="G70" s="6" t="n">
+        <v>53.334</v>
+      </c>
+      <c r="H70" s="6" t="n">
+        <v>56.038</v>
+      </c>
+      <c r="I70" s="6" t="n">
+        <v>56.923</v>
+      </c>
       <c r="J70" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3367,12 +3887,20 @@
         <v>-0.725</v>
       </c>
       <c r="E71" s="8" t="n">
-        <v>3.446</v>
-      </c>
-      <c r="F71" s="8" t="n"/>
-      <c r="G71" s="8" t="n"/>
-      <c r="H71" s="8" t="n"/>
-      <c r="I71" s="8" t="n"/>
+        <v>1.516409</v>
+      </c>
+      <c r="F71" s="8" t="n">
+        <v>53.599</v>
+      </c>
+      <c r="G71" s="8" t="n">
+        <v>52.418</v>
+      </c>
+      <c r="H71" s="8" t="n">
+        <v>56.453</v>
+      </c>
+      <c r="I71" s="8" t="n">
+        <v>55.327</v>
+      </c>
       <c r="J71" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3410,12 +3938,20 @@
         <v>1.581</v>
       </c>
       <c r="E72" s="6" t="n">
-        <v>6.083</v>
-      </c>
-      <c r="F72" s="6" t="n"/>
-      <c r="G72" s="6" t="n"/>
-      <c r="H72" s="6" t="n"/>
-      <c r="I72" s="6" t="n"/>
+        <v>5.366673</v>
+      </c>
+      <c r="F72" s="6" t="n">
+        <v>53.657</v>
+      </c>
+      <c r="G72" s="6" t="n">
+        <v>53.188</v>
+      </c>
+      <c r="H72" s="6" t="n">
+        <v>56.343</v>
+      </c>
+      <c r="I72" s="6" t="n">
+        <v>58.635</v>
+      </c>
       <c r="J72" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3453,12 +3989,20 @@
         <v>-0.1</v>
       </c>
       <c r="E73" s="8" t="n">
-        <v>7.984</v>
-      </c>
-      <c r="F73" s="8" t="n"/>
-      <c r="G73" s="8" t="n"/>
-      <c r="H73" s="8" t="n"/>
-      <c r="I73" s="8" t="n"/>
+        <v>4.421398</v>
+      </c>
+      <c r="F73" s="8" t="n">
+        <v>53.275</v>
+      </c>
+      <c r="G73" s="8" t="n">
+        <v>52.503</v>
+      </c>
+      <c r="H73" s="8" t="n">
+        <v>56.542</v>
+      </c>
+      <c r="I73" s="8" t="n">
+        <v>58.631</v>
+      </c>
       <c r="J73" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3496,12 +4040,20 @@
         <v>-0.075</v>
       </c>
       <c r="E74" s="6" t="n">
-        <v>8.397</v>
-      </c>
-      <c r="F74" s="6" t="n"/>
-      <c r="G74" s="6" t="n"/>
-      <c r="H74" s="6" t="n"/>
-      <c r="I74" s="6" t="n"/>
+        <v>1.028716</v>
+      </c>
+      <c r="F74" s="6" t="n">
+        <v>53.66</v>
+      </c>
+      <c r="G74" s="6" t="n">
+        <v>53.171</v>
+      </c>
+      <c r="H74" s="6" t="n">
+        <v>55.637</v>
+      </c>
+      <c r="I74" s="6" t="n">
+        <v>58.618</v>
+      </c>
       <c r="J74" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3539,12 +4091,20 @@
         <v>-0.912</v>
       </c>
       <c r="E75" s="8" t="n">
-        <v>5.601</v>
-      </c>
-      <c r="F75" s="8" t="n"/>
-      <c r="G75" s="8" t="n"/>
-      <c r="H75" s="8" t="n"/>
-      <c r="I75" s="8" t="n"/>
+        <v>-6.270722</v>
+      </c>
+      <c r="F75" s="8" t="n">
+        <v>53.919</v>
+      </c>
+      <c r="G75" s="8" t="n">
+        <v>52.305</v>
+      </c>
+      <c r="H75" s="8" t="n">
+        <v>55.171</v>
+      </c>
+      <c r="I75" s="8" t="n">
+        <v>56.93</v>
+      </c>
       <c r="J75" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3582,12 +4142,20 @@
         <v>0.599</v>
       </c>
       <c r="E76" s="6" t="n">
-        <v>6.445</v>
-      </c>
-      <c r="F76" s="6" t="n"/>
-      <c r="G76" s="6" t="n"/>
-      <c r="H76" s="6" t="n"/>
-      <c r="I76" s="6" t="n"/>
+        <v>1.757008</v>
+      </c>
+      <c r="F76" s="6" t="n">
+        <v>53.748</v>
+      </c>
+      <c r="G76" s="6" t="n">
+        <v>51.766</v>
+      </c>
+      <c r="H76" s="6" t="n">
+        <v>56.308</v>
+      </c>
+      <c r="I76" s="6" t="n">
+        <v>57.838</v>
+      </c>
       <c r="J76" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3625,12 +4193,20 @@
         <v>0.12</v>
       </c>
       <c r="E77" s="8" t="n">
-        <v>8.766</v>
-      </c>
-      <c r="F77" s="8" t="n"/>
-      <c r="G77" s="8" t="n"/>
-      <c r="H77" s="8" t="n"/>
-      <c r="I77" s="8" t="n"/>
+        <v>5.499725</v>
+      </c>
+      <c r="F77" s="8" t="n">
+        <v>54.197</v>
+      </c>
+      <c r="G77" s="8" t="n">
+        <v>51.267</v>
+      </c>
+      <c r="H77" s="8" t="n">
+        <v>56.346</v>
+      </c>
+      <c r="I77" s="8" t="n">
+        <v>57.973</v>
+      </c>
       <c r="J77" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3668,12 +4244,20 @@
         <v>-0.197</v>
       </c>
       <c r="E78" s="6" t="n">
-        <v>7.421</v>
-      </c>
-      <c r="F78" s="6" t="n"/>
-      <c r="G78" s="6" t="n"/>
-      <c r="H78" s="6" t="n"/>
-      <c r="I78" s="6" t="n"/>
+        <v>-3.207618</v>
+      </c>
+      <c r="F78" s="6" t="n">
+        <v>54.113</v>
+      </c>
+      <c r="G78" s="6" t="n">
+        <v>52.849</v>
+      </c>
+      <c r="H78" s="6" t="n">
+        <v>54.242</v>
+      </c>
+      <c r="I78" s="6" t="n">
+        <v>58.339</v>
+      </c>
       <c r="J78" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3711,12 +4295,20 @@
         <v>-0.996</v>
       </c>
       <c r="E79" s="8" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="F79" s="8" t="n"/>
-      <c r="G79" s="8" t="n"/>
-      <c r="H79" s="8" t="n"/>
-      <c r="I79" s="8" t="n"/>
+        <v>-9.104684000000001</v>
+      </c>
+      <c r="F79" s="8" t="n">
+        <v>54.517</v>
+      </c>
+      <c r="G79" s="8" t="n">
+        <v>49.958</v>
+      </c>
+      <c r="H79" s="8" t="n">
+        <v>53.966</v>
+      </c>
+      <c r="I79" s="8" t="n">
+        <v>56.714</v>
+      </c>
       <c r="J79" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3754,12 +4346,20 @@
         <v>-0.218</v>
       </c>
       <c r="E80" s="6" t="n">
-        <v>1.146</v>
-      </c>
-      <c r="F80" s="6" t="n"/>
-      <c r="G80" s="6" t="n"/>
-      <c r="H80" s="6" t="n"/>
-      <c r="I80" s="6" t="n"/>
+        <v>-4.042968</v>
+      </c>
+      <c r="F80" s="6" t="n">
+        <v>54.585</v>
+      </c>
+      <c r="G80" s="6" t="n">
+        <v>52.076</v>
+      </c>
+      <c r="H80" s="6" t="n">
+        <v>54.104</v>
+      </c>
+      <c r="I80" s="6" t="n">
+        <v>55.71</v>
+      </c>
       <c r="J80" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3797,12 +4397,20 @@
         <v>0.2</v>
       </c>
       <c r="E81" s="8" t="n">
-        <v>0.181</v>
-      </c>
-      <c r="F81" s="8" t="n"/>
-      <c r="G81" s="8" t="n"/>
-      <c r="H81" s="8" t="n"/>
-      <c r="I81" s="8" t="n"/>
+        <v>-1.807184</v>
+      </c>
+      <c r="F81" s="8" t="n">
+        <v>54.542</v>
+      </c>
+      <c r="G81" s="8" t="n">
+        <v>52.821</v>
+      </c>
+      <c r="H81" s="8" t="n">
+        <v>54.206</v>
+      </c>
+      <c r="I81" s="8" t="n">
+        <v>55.962</v>
+      </c>
       <c r="J81" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3840,12 +4448,20 @@
         <v>-0.320114</v>
       </c>
       <c r="E82" s="6" t="n">
-        <v>-1.043114</v>
-      </c>
-      <c r="F82" s="6" t="n"/>
-      <c r="G82" s="6" t="n"/>
-      <c r="H82" s="6" t="n"/>
-      <c r="I82" s="6" t="n"/>
+        <v>-2.203846</v>
+      </c>
+      <c r="F82" s="6" t="n">
+        <v>54.179614</v>
+      </c>
+      <c r="G82" s="6" t="n">
+        <v>50.676569</v>
+      </c>
+      <c r="H82" s="6" t="n">
+        <v>53.474536</v>
+      </c>
+      <c r="I82" s="6" t="n">
+        <v>56.239812</v>
+      </c>
       <c r="J82" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3883,12 +4499,20 @@
         <v>-1.486992</v>
       </c>
       <c r="E83" s="8" t="n">
-        <v>-1.805107</v>
-      </c>
-      <c r="F83" s="8" t="n"/>
-      <c r="G83" s="8" t="n"/>
-      <c r="H83" s="8" t="n"/>
-      <c r="I83" s="8" t="n"/>
+        <v>-1.41129</v>
+      </c>
+      <c r="F83" s="8" t="n">
+        <v>53.132812</v>
+      </c>
+      <c r="G83" s="8" t="n">
+        <v>50.317052</v>
+      </c>
+      <c r="H83" s="8" t="n">
+        <v>53.449466</v>
+      </c>
+      <c r="I83" s="8" t="n">
+        <v>53.576937</v>
+      </c>
       <c r="J83" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3926,12 +4550,20 @@
         <v>0.342203</v>
       </c>
       <c r="E84" s="6" t="n">
-        <v>-3.043904</v>
-      </c>
-      <c r="F84" s="6" t="n"/>
-      <c r="G84" s="6" t="n"/>
-      <c r="H84" s="6" t="n"/>
-      <c r="I84" s="6" t="n"/>
+        <v>-2.099311</v>
+      </c>
+      <c r="F84" s="6" t="n">
+        <v>52.989241</v>
+      </c>
+      <c r="G84" s="6" t="n">
+        <v>50.622791</v>
+      </c>
+      <c r="H84" s="6" t="n">
+        <v>53.085435</v>
+      </c>
+      <c r="I84" s="6" t="n">
+        <v>54.510294</v>
+      </c>
       <c r="J84" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3969,12 +4601,20 @@
         <v>-0.75157</v>
       </c>
       <c r="E85" s="8" t="n">
-        <v>-3.695474</v>
-      </c>
-      <c r="F85" s="8" t="n"/>
-      <c r="G85" s="8" t="n"/>
-      <c r="H85" s="8" t="n"/>
-      <c r="I85" s="8" t="n"/>
+        <v>-1.16407</v>
+      </c>
+      <c r="F85" s="8" t="n">
+        <v>52.885945</v>
+      </c>
+      <c r="G85" s="8" t="n">
+        <v>51.122903</v>
+      </c>
+      <c r="H85" s="8" t="n">
+        <v>52.604894</v>
+      </c>
+      <c r="I85" s="8" t="n">
+        <v>53.06938</v>
+      </c>
       <c r="J85" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4012,12 +4652,20 @@
         <v>-1.755021</v>
       </c>
       <c r="E86" s="6" t="n">
-        <v>-5.375495</v>
-      </c>
-      <c r="F86" s="6" t="n"/>
-      <c r="G86" s="6" t="n"/>
-      <c r="H86" s="6" t="n"/>
-      <c r="I86" s="6" t="n"/>
+        <v>-2.989536</v>
+      </c>
+      <c r="F86" s="6" t="n">
+        <v>51.576526</v>
+      </c>
+      <c r="G86" s="6" t="n">
+        <v>47.887594</v>
+      </c>
+      <c r="H86" s="6" t="n">
+        <v>51.522499</v>
+      </c>
+      <c r="I86" s="6" t="n">
+        <v>51.06508</v>
+      </c>
       <c r="J86" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4055,12 +4703,20 @@
         <v>0.920679</v>
       </c>
       <c r="E87" s="8" t="n">
-        <v>-3.542817</v>
-      </c>
-      <c r="F87" s="8" t="n"/>
-      <c r="G87" s="8" t="n"/>
-      <c r="H87" s="8" t="n"/>
-      <c r="I87" s="8" t="n"/>
+        <v>3.14829</v>
+      </c>
+      <c r="F87" s="8" t="n">
+        <v>51.978727</v>
+      </c>
+      <c r="G87" s="8" t="n">
+        <v>48.998174</v>
+      </c>
+      <c r="H87" s="8" t="n">
+        <v>52.32137</v>
+      </c>
+      <c r="I87" s="8" t="n">
+        <v>52.248185</v>
+      </c>
       <c r="J87" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4098,12 +4754,20 @@
         <v>-0.421547</v>
       </c>
       <c r="E88" s="6" t="n">
-        <v>-4.563364</v>
-      </c>
-      <c r="F88" s="6" t="n"/>
-      <c r="G88" s="6" t="n"/>
-      <c r="H88" s="6" t="n"/>
-      <c r="I88" s="6" t="n"/>
+        <v>-1.75256</v>
+      </c>
+      <c r="F88" s="6" t="n">
+        <v>51.622676</v>
+      </c>
+      <c r="G88" s="6" t="n">
+        <v>49.201964</v>
+      </c>
+      <c r="H88" s="6" t="n">
+        <v>51.863878</v>
+      </c>
+      <c r="I88" s="6" t="n">
+        <v>51.688565</v>
+      </c>
       <c r="J88" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4141,12 +4805,20 @@
         <v>0.411983</v>
       </c>
       <c r="E89" s="8" t="n">
-        <v>-4.27138</v>
-      </c>
-      <c r="F89" s="8" t="n"/>
-      <c r="G89" s="8" t="n"/>
-      <c r="H89" s="8" t="n"/>
-      <c r="I89" s="8" t="n"/>
+        <v>0.537234</v>
+      </c>
+      <c r="F89" s="8" t="n">
+        <v>50.91615</v>
+      </c>
+      <c r="G89" s="8" t="n">
+        <v>48.748217</v>
+      </c>
+      <c r="H89" s="8" t="n">
+        <v>52.017722</v>
+      </c>
+      <c r="I89" s="8" t="n">
+        <v>52.92183</v>
+      </c>
       <c r="J89" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4184,12 +4856,20 @@
         <v>-0.521713</v>
       </c>
       <c r="E90" s="6" t="n">
-        <v>-4.596093</v>
-      </c>
-      <c r="F90" s="6" t="n"/>
-      <c r="G90" s="6" t="n"/>
-      <c r="H90" s="6" t="n"/>
-      <c r="I90" s="6" t="n"/>
+        <v>-0.606911</v>
+      </c>
+      <c r="F90" s="6" t="n">
+        <v>51.362162</v>
+      </c>
+      <c r="G90" s="6" t="n">
+        <v>48.098086</v>
+      </c>
+      <c r="H90" s="6" t="n">
+        <v>52.463376</v>
+      </c>
+      <c r="I90" s="6" t="n">
+        <v>51.487236</v>
+      </c>
       <c r="J90" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4227,12 +4907,20 @@
         <v>-1.257464</v>
       </c>
       <c r="E91" s="8" t="n">
-        <v>-4.857557</v>
-      </c>
-      <c r="F91" s="8" t="n"/>
-      <c r="G91" s="8" t="n"/>
-      <c r="H91" s="8" t="n"/>
-      <c r="I91" s="8" t="n"/>
+        <v>-0.624376</v>
+      </c>
+      <c r="F91" s="8" t="n">
+        <v>50.547437</v>
+      </c>
+      <c r="G91" s="8" t="n">
+        <v>46.76653</v>
+      </c>
+      <c r="H91" s="8" t="n">
+        <v>50.564832</v>
+      </c>
+      <c r="I91" s="8" t="n">
+        <v>50.36792</v>
+      </c>
       <c r="J91" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4270,12 +4958,20 @@
         <v>-0.779626</v>
       </c>
       <c r="E92" s="6" t="n">
-        <v>-5.419183</v>
-      </c>
-      <c r="F92" s="6" t="n"/>
-      <c r="G92" s="6" t="n"/>
-      <c r="H92" s="6" t="n"/>
-      <c r="I92" s="6" t="n"/>
+        <v>-1.060847</v>
+      </c>
+      <c r="F92" s="6" t="n">
+        <v>50.202057</v>
+      </c>
+      <c r="G92" s="6" t="n">
+        <v>46.853136</v>
+      </c>
+      <c r="H92" s="6" t="n">
+        <v>49.188614</v>
+      </c>
+      <c r="I92" s="6" t="n">
+        <v>49.517803</v>
+      </c>
       <c r="J92" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4313,12 +5009,20 @@
         <v>-0.648362</v>
       </c>
       <c r="E93" s="8" t="n">
-        <v>-6.267545</v>
-      </c>
-      <c r="F93" s="8" t="n"/>
-      <c r="G93" s="8" t="n"/>
-      <c r="H93" s="8" t="n"/>
-      <c r="I93" s="8" t="n"/>
+        <v>-1.507667</v>
+      </c>
+      <c r="F93" s="8" t="n">
+        <v>48.690879</v>
+      </c>
+      <c r="G93" s="8" t="n">
+        <v>46.683058</v>
+      </c>
+      <c r="H93" s="8" t="n">
+        <v>47.264022</v>
+      </c>
+      <c r="I93" s="8" t="n">
+        <v>49.820923</v>
+      </c>
       <c r="J93" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4356,12 +5060,20 @@
         <v>0.032747</v>
       </c>
       <c r="E94" s="6" t="n">
-        <v>-5.914683</v>
-      </c>
-      <c r="F94" s="6" t="n"/>
-      <c r="G94" s="6" t="n"/>
-      <c r="H94" s="6" t="n"/>
-      <c r="I94" s="6" t="n"/>
+        <v>0.579012</v>
+      </c>
+      <c r="F94" s="6" t="n">
+        <v>49.843553</v>
+      </c>
+      <c r="G94" s="6" t="n">
+        <v>46.355094</v>
+      </c>
+      <c r="H94" s="6" t="n">
+        <v>46.755586</v>
+      </c>
+      <c r="I94" s="6" t="n">
+        <v>49.687044</v>
+      </c>
       <c r="J94" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4399,12 +5111,20 @@
         <v>-0.098581</v>
       </c>
       <c r="E95" s="8" t="n">
-        <v>-4.526271</v>
-      </c>
-      <c r="F95" s="8" t="n"/>
-      <c r="G95" s="8" t="n"/>
-      <c r="H95" s="8" t="n"/>
-      <c r="I95" s="8" t="n"/>
+        <v>2.30939</v>
+      </c>
+      <c r="F95" s="8" t="n">
+        <v>49.228847</v>
+      </c>
+      <c r="G95" s="8" t="n">
+        <v>47.481149</v>
+      </c>
+      <c r="H95" s="8" t="n">
+        <v>47.550991</v>
+      </c>
+      <c r="I95" s="8" t="n">
+        <v>49.1228</v>
+      </c>
       <c r="J95" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4442,12 +5162,20 @@
         <v>0.344711</v>
       </c>
       <c r="E96" s="6" t="n">
-        <v>-4.523763</v>
-      </c>
-      <c r="F96" s="6" t="n"/>
-      <c r="G96" s="6" t="n"/>
-      <c r="H96" s="6" t="n"/>
-      <c r="I96" s="6" t="n"/>
+        <v>0.059169</v>
+      </c>
+      <c r="F96" s="6" t="n">
+        <v>49.341468</v>
+      </c>
+      <c r="G96" s="6" t="n">
+        <v>47.049596</v>
+      </c>
+      <c r="H96" s="6" t="n">
+        <v>47.151559</v>
+      </c>
+      <c r="I96" s="6" t="n">
+        <v>50.110607</v>
+      </c>
       <c r="J96" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4485,12 +5213,20 @@
         <v>0.334323</v>
       </c>
       <c r="E97" s="8" t="n">
-        <v>-3.437869</v>
-      </c>
-      <c r="F97" s="8" t="n"/>
-      <c r="G97" s="8" t="n"/>
-      <c r="H97" s="8" t="n"/>
-      <c r="I97" s="8" t="n"/>
+        <v>1.938422</v>
+      </c>
+      <c r="F97" s="8" t="n">
+        <v>49.210834</v>
+      </c>
+      <c r="G97" s="8" t="n">
+        <v>46.197266</v>
+      </c>
+      <c r="H97" s="8" t="n">
+        <v>48.49971</v>
+      </c>
+      <c r="I97" s="8" t="n">
+        <v>50.381451</v>
+      </c>
       <c r="J97" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4528,12 +5264,20 @@
         <v>0.016742</v>
       </c>
       <c r="E98" s="6" t="n">
-        <v>-1.666106</v>
-      </c>
-      <c r="F98" s="6" t="n"/>
-      <c r="G98" s="6" t="n"/>
-      <c r="H98" s="6" t="n"/>
-      <c r="I98" s="6" t="n"/>
+        <v>3.250656</v>
+      </c>
+      <c r="F98" s="6" t="n">
+        <v>49.155734</v>
+      </c>
+      <c r="G98" s="6" t="n">
+        <v>46.493502</v>
+      </c>
+      <c r="H98" s="6" t="n">
+        <v>48.186482</v>
+      </c>
+      <c r="I98" s="6" t="n">
+        <v>50.543125</v>
+      </c>
       <c r="J98" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4571,12 +5315,20 @@
         <v>-0.807123</v>
       </c>
       <c r="E99" s="8" t="n">
-        <v>-3.393907</v>
-      </c>
-      <c r="F99" s="8" t="n"/>
-      <c r="G99" s="8" t="n"/>
-      <c r="H99" s="8" t="n"/>
-      <c r="I99" s="8" t="n"/>
+        <v>-3.270739</v>
+      </c>
+      <c r="F99" s="8" t="n">
+        <v>48.83249</v>
+      </c>
+      <c r="G99" s="8" t="n">
+        <v>45.847665</v>
+      </c>
+      <c r="H99" s="8" t="n">
+        <v>47.870006</v>
+      </c>
+      <c r="I99" s="8" t="n">
+        <v>49.230472</v>
+      </c>
       <c r="J99" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4614,12 +5366,20 @@
         <v>-0.209162</v>
       </c>
       <c r="E100" s="6" t="n">
-        <v>-3.181522</v>
-      </c>
-      <c r="F100" s="6" t="n"/>
-      <c r="G100" s="6" t="n"/>
-      <c r="H100" s="6" t="n"/>
-      <c r="I100" s="6" t="n"/>
+        <v>0.358984</v>
+      </c>
+      <c r="F100" s="6" t="n">
+        <v>48.233571</v>
+      </c>
+      <c r="G100" s="6" t="n">
+        <v>46.046766</v>
+      </c>
+      <c r="H100" s="6" t="n">
+        <v>47.73379</v>
+      </c>
+      <c r="I100" s="6" t="n">
+        <v>49.08107</v>
+      </c>
       <c r="J100" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4657,12 +5417,20 @@
         <v>-0.154983</v>
       </c>
       <c r="E101" s="8" t="n">
-        <v>-3.74849</v>
-      </c>
-      <c r="F101" s="8" t="n"/>
-      <c r="G101" s="8" t="n"/>
-      <c r="H101" s="8" t="n"/>
-      <c r="I101" s="8" t="n"/>
+        <v>-1.043436</v>
+      </c>
+      <c r="F101" s="8" t="n">
+        <v>48.199845</v>
+      </c>
+      <c r="G101" s="8" t="n">
+        <v>45.064614</v>
+      </c>
+      <c r="H101" s="8" t="n">
+        <v>47.725481</v>
+      </c>
+      <c r="I101" s="8" t="n">
+        <v>48.962478</v>
+      </c>
       <c r="J101" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4700,12 +5468,20 @@
         <v>-0.14389</v>
       </c>
       <c r="E102" s="6" t="n">
-        <v>-3.370667</v>
-      </c>
-      <c r="F102" s="6" t="n"/>
-      <c r="G102" s="6" t="n"/>
-      <c r="H102" s="6" t="n"/>
-      <c r="I102" s="6" t="n"/>
+        <v>0.662073</v>
+      </c>
+      <c r="F102" s="6" t="n">
+        <v>48.032404</v>
+      </c>
+      <c r="G102" s="6" t="n">
+        <v>45.501564</v>
+      </c>
+      <c r="H102" s="6" t="n">
+        <v>47.135756</v>
+      </c>
+      <c r="I102" s="6" t="n">
+        <v>48.93954</v>
+      </c>
       <c r="J102" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4743,12 +5519,20 @@
         <v>0.791872</v>
       </c>
       <c r="E103" s="8" t="n">
-        <v>-1.321332</v>
-      </c>
-      <c r="F103" s="8" t="n"/>
-      <c r="G103" s="8" t="n"/>
-      <c r="H103" s="8" t="n"/>
-      <c r="I103" s="8" t="n"/>
+        <v>3.92445</v>
+      </c>
+      <c r="F103" s="8" t="n">
+        <v>48.432033</v>
+      </c>
+      <c r="G103" s="8" t="n">
+        <v>46.529004</v>
+      </c>
+      <c r="H103" s="8" t="n">
+        <v>48.708475</v>
+      </c>
+      <c r="I103" s="8" t="n">
+        <v>49.466133</v>
+      </c>
       <c r="J103" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4786,12 +5570,20 @@
         <v>-0.353837</v>
       </c>
       <c r="E104" s="6" t="n">
-        <v>-0.895543</v>
-      </c>
-      <c r="F104" s="6" t="n"/>
-      <c r="G104" s="6" t="n"/>
-      <c r="H104" s="6" t="n"/>
-      <c r="I104" s="6" t="n"/>
+        <v>0.821345</v>
+      </c>
+      <c r="F104" s="6" t="n">
+        <v>47.946339</v>
+      </c>
+      <c r="G104" s="6" t="n">
+        <v>47.83974</v>
+      </c>
+      <c r="H104" s="6" t="n">
+        <v>49.009558</v>
+      </c>
+      <c r="I104" s="6" t="n">
+        <v>48.502866</v>
+      </c>
       <c r="J104" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4829,12 +5621,20 @@
         <v>-0.085068</v>
       </c>
       <c r="E105" s="8" t="n">
-        <v>-0.332249</v>
-      </c>
-      <c r="F105" s="8" t="n"/>
-      <c r="G105" s="8" t="n"/>
-      <c r="H105" s="8" t="n"/>
-      <c r="I105" s="8" t="n"/>
+        <v>1.13274</v>
+      </c>
+      <c r="F105" s="8" t="n">
+        <v>48.327254</v>
+      </c>
+      <c r="G105" s="8" t="n">
+        <v>48.111931</v>
+      </c>
+      <c r="H105" s="8" t="n">
+        <v>49.031304</v>
+      </c>
+      <c r="I105" s="8" t="n">
+        <v>48.076703</v>
+      </c>
       <c r="J105" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4872,12 +5672,20 @@
         <v>-0.131213</v>
       </c>
       <c r="E106" s="6" t="n">
-        <v>-0.496211</v>
-      </c>
-      <c r="F106" s="6" t="n"/>
-      <c r="G106" s="6" t="n"/>
-      <c r="H106" s="6" t="n"/>
-      <c r="I106" s="6" t="n"/>
+        <v>-0.336063</v>
+      </c>
+      <c r="F106" s="6" t="n">
+        <v>47.783735</v>
+      </c>
+      <c r="G106" s="6" t="n">
+        <v>47.739796</v>
+      </c>
+      <c r="H106" s="6" t="n">
+        <v>48.310078</v>
+      </c>
+      <c r="I106" s="6" t="n">
+        <v>48.484834</v>
+      </c>
       <c r="J106" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4915,12 +5723,20 @@
         <v>-0.069019</v>
       </c>
       <c r="E107" s="8" t="n">
-        <v>-0.466649</v>
-      </c>
-      <c r="F107" s="8" t="n"/>
-      <c r="G107" s="8" t="n"/>
-      <c r="H107" s="8" t="n"/>
-      <c r="I107" s="8" t="n"/>
+        <v>0.058732</v>
+      </c>
+      <c r="F107" s="8" t="n">
+        <v>48.03239</v>
+      </c>
+      <c r="G107" s="8" t="n">
+        <v>46.252625</v>
+      </c>
+      <c r="H107" s="8" t="n">
+        <v>48.91357</v>
+      </c>
+      <c r="I107" s="8" t="n">
+        <v>48.212931</v>
+      </c>
       <c r="J107" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4958,12 +5774,20 @@
         <v>0.046638</v>
       </c>
       <c r="E108" s="6" t="n">
-        <v>-0.764721</v>
-      </c>
-      <c r="F108" s="6" t="n"/>
-      <c r="G108" s="6" t="n"/>
-      <c r="H108" s="6" t="n"/>
-      <c r="I108" s="6" t="n"/>
+        <v>-0.60195</v>
+      </c>
+      <c r="F108" s="6" t="n">
+        <v>47.907922</v>
+      </c>
+      <c r="G108" s="6" t="n">
+        <v>47.126658</v>
+      </c>
+      <c r="H108" s="6" t="n">
+        <v>48.257084</v>
+      </c>
+      <c r="I108" s="6" t="n">
+        <v>48.529883</v>
+      </c>
       <c r="J108" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -5001,12 +5825,20 @@
         <v>0.029301</v>
       </c>
       <c r="E109" s="8" t="n">
-        <v>-1.069745</v>
-      </c>
-      <c r="F109" s="8" t="n"/>
-      <c r="G109" s="8" t="n"/>
-      <c r="H109" s="8" t="n"/>
-      <c r="I109" s="8" t="n"/>
+        <v>-0.608084</v>
+      </c>
+      <c r="F109" s="8" t="n">
+        <v>47.997733</v>
+      </c>
+      <c r="G109" s="8" t="n">
+        <v>47.498528</v>
+      </c>
+      <c r="H109" s="8" t="n">
+        <v>48.000377</v>
+      </c>
+      <c r="I109" s="8" t="n">
+        <v>48.608038</v>
+      </c>
       <c r="J109" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>

</xml_diff>